<commit_message>
2026 NY envelopes 2026 PM3D sample randomizations
</commit_message>
<xml_diff>
--- a/data/B4I_2026/26NY_POI.xlsx
+++ b/data/B4I_2026/26NY_POI.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\garrett.raymon\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pth7\Documents\Intercrop JLJ\B4I\B4I_hyde\data\B4I_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{062A806F-9B64-4C5C-BAA9-CA5610A1597D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B4F3934-9F84-4F43-AF63-456095FB54AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{6B20FC54-A660-4868-91E2-CC4FD6A289D5}"/>
+    <workbookView xWindow="2925" yWindow="1080" windowWidth="28965" windowHeight="19290" xr2:uid="{6B20FC54-A660-4868-91E2-CC4FD6A289D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$G$7</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,9 +34,6 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -791,7 +789,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -799,15 +797,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1142,152 +1157,160 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E70D119A-6C72-4B0B-A2CD-1DC16CF5078F}">
-  <dimension ref="A1:F233"/>
+  <dimension ref="A1:G233"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="3" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
+      <c r="G1" s="3"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="3">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3">
         <v>58.8</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="3">
         <f>D2/C2</f>
         <v>58.8</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="3">
-        <v>1</v>
-      </c>
-      <c r="D3" s="3">
+      <c r="C3" s="5">
+        <v>1</v>
+      </c>
+      <c r="D3" s="5">
         <v>562</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="5">
         <v>70.3</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="5">
         <v>117</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
         <v>236</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="5">
         <v>0</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="5">
         <v>528</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="5">
         <v>66</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="5">
         <v>110</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+      <c r="G4" s="3"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="3">
-        <v>2</v>
-      </c>
-      <c r="D5" s="3">
+      <c r="C5" s="5">
+        <v>2</v>
+      </c>
+      <c r="D5" s="5">
         <v>692</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="5">
         <v>76.900000000000006</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="5">
         <v>128</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+      <c r="G5" s="3"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="3">
-        <v>2</v>
-      </c>
-      <c r="D6" s="3">
+      <c r="C6" s="5">
+        <v>2</v>
+      </c>
+      <c r="D6" s="5">
         <v>638</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="5">
         <v>70.8</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="5">
         <v>118</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+      <c r="G6" s="3"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
         <v>237</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="5">
         <v>0</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="5">
         <v>362</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="5">
         <v>60.2</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="5">
         <v>100.3</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="3"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>238</v>
       </c>
@@ -1301,11 +1324,11 @@
         <v>61.6</v>
       </c>
       <c r="E8">
-        <f t="shared" ref="E3:E66" si="0">D8/C8</f>
+        <f t="shared" ref="E8:E66" si="0">D8/C8</f>
         <v>61.6</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>6</v>
       </c>
@@ -1323,7 +1346,7 @@
         <v>67.099999999999994</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>7</v>
       </c>
@@ -1341,7 +1364,7 @@
         <v>82.1</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>240</v>
       </c>
@@ -1359,7 +1382,7 @@
         <v>61.9</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>8</v>
       </c>
@@ -1377,7 +1400,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>273</v>
       </c>
@@ -1395,7 +1418,7 @@
         <v>57.6</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>274</v>
       </c>
@@ -1413,7 +1436,7 @@
         <v>61.6</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>9</v>
       </c>
@@ -1431,7 +1454,7 @@
         <v>64.8</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>275</v>
       </c>
@@ -5362,5 +5385,6 @@
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>